<commit_message>
B1: cardápios de CCG Floripa, Jogasampa e Tubaleria a partir de prints
Pedido do autor: incluir os prints de cardápio (fotos do Maps e destaque
do Instagram) esquecidos no envio anterior. Planilha com 37 casas, resumo,
estatística, site e Notion atualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/[B1] Estabelecimentos e cardapios/estabelecimentos/4_estatistica_descritiva/B1_estatistica_descritiva_geral.xlsx
+++ b/dados/[B1] Estabelecimentos e cardapios/estabelecimentos/4_estatistica_descritiva/B1_estatistica_descritiva_geral.xlsx
@@ -6306,7 +6306,9 @@
       <c r="AH18" s="14" t="n"/>
       <c r="AI18" s="14" t="n"/>
       <c r="AJ18" s="14" t="n"/>
-      <c r="AK18" s="7" t="n"/>
+      <c r="AK18" s="7" t="n">
+        <v>362</v>
+      </c>
       <c r="AL18" s="7" t="n">
         <v>10</v>
       </c>
@@ -8836,9 +8838,13 @@
       <c r="X36" s="12" t="n">
         <v>0.00233</v>
       </c>
-      <c r="Y36" s="7" t="n"/>
+      <c r="Y36" s="7" t="n">
+        <v>7</v>
+      </c>
       <c r="Z36" s="14" t="n"/>
-      <c r="AA36" s="14" t="n"/>
+      <c r="AA36" s="14" t="n">
+        <v>6</v>
+      </c>
       <c r="AB36" s="14" t="n"/>
       <c r="AC36" s="14" t="n"/>
       <c r="AD36" s="14" t="n"/>
@@ -8846,7 +8852,9 @@
       <c r="AF36" s="14" t="n"/>
       <c r="AG36" s="14" t="n"/>
       <c r="AH36" s="14" t="n"/>
-      <c r="AI36" s="14" t="n"/>
+      <c r="AI36" s="14" t="n">
+        <v>6</v>
+      </c>
       <c r="AJ36" s="14" t="n"/>
       <c r="AK36" s="7" t="n">
         <v>331</v>
@@ -8861,9 +8869,11 @@
         <v>1</v>
       </c>
       <c r="AO36" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP36" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AP36" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="AQ36" s="4" t="n">
         <v>0</v>
       </c>
@@ -9676,15 +9686,23 @@
         <v>41.6</v>
       </c>
       <c r="X42" s="12" t="n"/>
-      <c r="Y42" s="7" t="n"/>
+      <c r="Y42" s="7" t="n">
+        <v>29</v>
+      </c>
       <c r="Z42" s="14" t="n"/>
       <c r="AA42" s="14" t="n"/>
-      <c r="AB42" s="14" t="n"/>
+      <c r="AB42" s="14" t="n">
+        <v>38</v>
+      </c>
       <c r="AC42" s="14" t="n"/>
       <c r="AD42" s="14" t="n"/>
       <c r="AE42" s="14" t="n"/>
-      <c r="AF42" s="14" t="n"/>
-      <c r="AG42" s="14" t="n"/>
+      <c r="AF42" s="14" t="n">
+        <v>48</v>
+      </c>
+      <c r="AG42" s="14" t="n">
+        <v>35</v>
+      </c>
       <c r="AH42" s="14" t="n"/>
       <c r="AI42" s="14" t="n"/>
       <c r="AJ42" s="14" t="n"/>
@@ -9697,9 +9715,11 @@
         <v>0</v>
       </c>
       <c r="AO42" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP42" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AP42" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="AQ42" s="4" t="n">
         <v>0</v>
       </c>
@@ -10871,15 +10891,23 @@
       <c r="X51" s="12" t="n">
         <v>0.03043</v>
       </c>
-      <c r="Y51" s="7" t="n"/>
+      <c r="Y51" s="7" t="n">
+        <v>9</v>
+      </c>
       <c r="Z51" s="14" t="n"/>
       <c r="AA51" s="14" t="n"/>
-      <c r="AB51" s="14" t="n"/>
+      <c r="AB51" s="14" t="n">
+        <v>36</v>
+      </c>
       <c r="AC51" s="14" t="n"/>
       <c r="AD51" s="14" t="n"/>
       <c r="AE51" s="14" t="n"/>
-      <c r="AF51" s="14" t="n"/>
-      <c r="AG51" s="14" t="n"/>
+      <c r="AF51" s="14" t="n">
+        <v>36</v>
+      </c>
+      <c r="AG51" s="14" t="n">
+        <v>54</v>
+      </c>
       <c r="AH51" s="14" t="n"/>
       <c r="AI51" s="14" t="n"/>
       <c r="AJ51" s="14" t="n"/>
@@ -10894,9 +10922,11 @@
         <v>0</v>
       </c>
       <c r="AO51" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP51" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AP51" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="AQ51" s="4" t="n">
         <v>0</v>
       </c>

</xml_diff>